<commit_message>
Add question 1 submission verification workflow
</commit_message>
<xml_diff>
--- a/output/question_1/q1_results.xlsx
+++ b/output/question_1/q1_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="345">
   <si>
     <t>index</t>
   </si>
@@ -979,6 +979,15 @@
     <t>plan_A_max_balance_residual</t>
   </si>
   <si>
+    <t>plan_A_max_soc_recurrence_residual</t>
+  </si>
+  <si>
+    <t>plan_A_max_lp_ub_violation</t>
+  </si>
+  <si>
+    <t>plan_A_max_lp_eq_residual</t>
+  </si>
+  <si>
     <t>plan_B_cost_yuan</t>
   </si>
   <si>
@@ -1001,6 +1010,15 @@
   </si>
   <si>
     <t>plan_B_max_balance_residual</t>
+  </si>
+  <si>
+    <t>plan_B_max_soc_recurrence_residual</t>
+  </si>
+  <si>
+    <t>plan_B_max_lp_ub_violation</t>
+  </si>
+  <si>
+    <t>plan_B_max_lp_eq_residual</t>
   </si>
   <si>
     <t>cost_saving_A_vs_no_storage_yuan</t>
@@ -10365,7 +10383,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -10461,7 +10479,7 @@
         <v>320</v>
       </c>
       <c r="B12">
-        <v>35126.94858928965</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -10469,7 +10487,7 @@
         <v>321</v>
       </c>
       <c r="B13">
-        <v>59482.69899835392</v>
+        <v>3.183231456205249E-12</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -10477,7 +10495,7 @@
         <v>322</v>
       </c>
       <c r="B14">
-        <v>20740.66613168725</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -10485,7 +10503,7 @@
         <v>323</v>
       </c>
       <c r="B15">
-        <v>16799.93956666668</v>
+        <v>35126.94858928965</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -10493,7 +10511,7 @@
         <v>324</v>
       </c>
       <c r="B16">
-        <v>1.74347450057313E-11</v>
+        <v>59482.69899835392</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -10501,7 +10519,7 @@
         <v>325</v>
       </c>
       <c r="B17">
-        <v>140</v>
+        <v>20740.66613168725</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -10509,7 +10527,7 @@
         <v>326</v>
       </c>
       <c r="B18">
-        <v>902.6919667008649</v>
+        <v>16799.93956666668</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -10517,7 +10535,7 @@
         <v>327</v>
       </c>
       <c r="B19">
-        <v>1.13686837721616E-13</v>
+        <v>1.74347450057313E-11</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -10525,7 +10543,7 @@
         <v>328</v>
       </c>
       <c r="B20">
-        <v>12925.09800155701</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -10533,7 +10551,7 @@
         <v>329</v>
       </c>
       <c r="B21">
-        <v>12925.09800155701</v>
+        <v>902.6919667008649</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -10541,15 +10559,63 @@
         <v>330</v>
       </c>
       <c r="B22">
-        <v>333.3333333676854</v>
+        <v>1.13686837721616E-13</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>331</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
         <v>332</v>
+      </c>
+      <c r="B24">
+        <v>2.160049916710705E-12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>333</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>334</v>
+      </c>
+      <c r="B26">
+        <v>12925.09800155701</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>335</v>
+      </c>
+      <c r="B27">
+        <v>12925.09800155701</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>336</v>
+      </c>
+      <c r="B28">
+        <v>333.3333333676854</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>337</v>
+      </c>
+      <c r="B29" t="s">
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -10587,7 +10653,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B2">
         <v>4500.000000000009</v>
@@ -10610,7 +10676,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="B3">
         <v>833.3333333333333</v>
@@ -10633,7 +10699,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="B4">
         <v>4787.964288065841</v>
@@ -10656,7 +10722,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="B5">
         <v>5286.035176954735</v>
@@ -10679,7 +10745,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="B6">
         <v>1.010549668636587E-11</v>
@@ -10702,7 +10768,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="B7">
         <v>5333.333333333529</v>

</xml_diff>